<commit_message>
Daily slate 2026-06-14 [auto]
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-06-11.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-06-11.xlsx
@@ -471,16 +471,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="E2" t="n">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="F2" t="n">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="G2" t="n">
-        <v>56.6</v>
+        <v>56.7</v>
       </c>
     </row>
     <row r="3">
@@ -500,16 +500,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="E3" t="n">
         <v>152</v>
       </c>
       <c r="F3" t="n">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="G3" t="n">
-        <v>53.3</v>
+        <v>52.4</v>
       </c>
     </row>
     <row r="4">
@@ -529,16 +529,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="E4" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="F4" t="n">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="G4" t="n">
-        <v>36</v>
+        <v>37.8</v>
       </c>
     </row>
     <row r="5">
@@ -726,16 +726,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>616</v>
+        <v>704</v>
       </c>
       <c r="E11" t="n">
-        <v>421</v>
+        <v>476</v>
       </c>
       <c r="F11" t="n">
-        <v>195</v>
+        <v>228</v>
       </c>
       <c r="G11" t="n">
-        <v>68.3</v>
+        <v>67.59999999999999</v>
       </c>
     </row>
     <row r="12">
@@ -755,16 +755,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="E12" t="n">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="F12" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G12" t="n">
-        <v>59.1</v>
+        <v>59.9</v>
       </c>
     </row>
     <row r="13">
@@ -784,16 +784,16 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E13" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F13" t="n">
         <v>42</v>
       </c>
       <c r="G13" t="n">
-        <v>49.4</v>
+        <v>50</v>
       </c>
     </row>
     <row r="14">
@@ -813,16 +813,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>222</v>
+        <v>236</v>
       </c>
       <c r="E14" t="n">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="F14" t="n">
-        <v>155</v>
+        <v>165</v>
       </c>
       <c r="G14" t="n">
-        <v>30.2</v>
+        <v>30.1</v>
       </c>
     </row>
     <row r="15">
@@ -842,16 +842,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>355</v>
+        <v>371</v>
       </c>
       <c r="E15" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="F15" t="n">
-        <v>257</v>
+        <v>269</v>
       </c>
       <c r="G15" t="n">
-        <v>27.6</v>
+        <v>27.5</v>
       </c>
     </row>
     <row r="16">
@@ -871,16 +871,16 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="E16" t="n">
         <v>90</v>
       </c>
       <c r="F16" t="n">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="G16" t="n">
-        <v>28.1</v>
+        <v>28</v>
       </c>
     </row>
     <row r="17">
@@ -900,16 +900,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>2177</v>
+        <v>2520</v>
       </c>
       <c r="E17" t="n">
-        <v>474</v>
+        <v>562</v>
       </c>
       <c r="F17" t="n">
-        <v>1703</v>
+        <v>1958</v>
       </c>
       <c r="G17" t="n">
-        <v>21.8</v>
+        <v>22.3</v>
       </c>
     </row>
   </sheetData>
@@ -1519,58 +1519,58 @@
         <v>194</v>
       </c>
       <c r="D7" t="n">
-        <v>68.3</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="E7" t="n">
-        <v>616</v>
+        <v>704</v>
       </c>
       <c r="F7" t="n">
-        <v>59.1</v>
+        <v>59.9</v>
       </c>
       <c r="G7" t="n">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="H7" t="n">
-        <v>49.4</v>
+        <v>50</v>
       </c>
       <c r="I7" t="n">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="J7" t="n">
-        <v>30.2</v>
+        <v>30.1</v>
       </c>
       <c r="K7" t="n">
-        <v>222</v>
+        <v>236</v>
       </c>
       <c r="L7" t="n">
-        <v>27.6</v>
+        <v>27.5</v>
       </c>
       <c r="M7" t="n">
-        <v>355</v>
+        <v>371</v>
       </c>
       <c r="N7" t="n">
-        <v>28.1</v>
+        <v>28</v>
       </c>
       <c r="O7" t="n">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="P7" t="n">
-        <v>21.8</v>
+        <v>22.3</v>
       </c>
       <c r="Q7" t="n">
-        <v>2177</v>
+        <v>2520</v>
       </c>
       <c r="R7" t="n">
-        <v>56.6</v>
+        <v>56.7</v>
       </c>
       <c r="S7" t="n">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="T7" t="n">
-        <v>36</v>
+        <v>37.8</v>
       </c>
       <c r="U7" t="n">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="W7" t="n">
         <v>0</v>
@@ -1582,10 +1582,10 @@
         <v>397</v>
       </c>
       <c r="Z7" t="n">
-        <v>53.3</v>
+        <v>52.4</v>
       </c>
       <c r="AA7" t="n">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="AB7" t="n">
         <v>0</v>

</xml_diff>